<commit_message>
Update KB Tracker fallback data after manual verification pass
Tested KB Tracker level-review flow end-to-end; everything working as expected.
</commit_message>
<xml_diff>
--- a/sample_data/KB_Updated.xlsx
+++ b/sample_data/KB_Updated.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6648" uniqueCount="1908">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6648" uniqueCount="1907">
   <si>
     <t>module_id</t>
   </si>
@@ -185,11 +185,11 @@
     <t>active</t>
   </si>
   <si>
-    <t xml:space="preserve">1 [APPROVED] - Need to change the Ad-Hoc
-2 [APPROVED] - Increase the percentage to 30 to 50%  check
-3 [APPROVED] - 
-4 [APPROVED] - 
-5 [APPROVED] - </t>
+    <t xml:space="preserve">1 [APPROVED] - 
+2 [PENDING] - 
+3 [PENDING] - 
+4 [PENDING] - 
+5 [PENDING] - </t>
   </si>
   <si>
     <t xml:space="preserve">• Is there a defined slot-booking mechanism for inbound vehicles? What % arrive within their booked slot?
@@ -7532,9 +7532,6 @@
   </si>
   <si>
     <t>review_status</t>
-  </si>
-  <si>
-    <t>Closed</t>
   </si>
   <si>
     <t>Needs review</t>
@@ -51725,7 +51722,7 @@
         <v>272</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I3" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51765,7 +51762,7 @@
         <v>281</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I4" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51805,7 +51802,7 @@
         <v>292</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I5" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51845,7 +51842,7 @@
         <v>301</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I6" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51885,7 +51882,7 @@
         <v>312</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I7" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51925,7 +51922,7 @@
         <v>409</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I8" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -51965,7 +51962,7 @@
         <v>322</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I9" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52005,7 +52002,7 @@
         <v>337</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I10" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52045,7 +52042,7 @@
         <v>350</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I11" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52085,7 +52082,7 @@
         <v>359</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I12" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52125,7 +52122,7 @@
         <v>368</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I13" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52165,7 +52162,7 @@
         <v>382</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I14" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52205,7 +52202,7 @@
         <v>391</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I15" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52245,7 +52242,7 @@
         <v>400</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I16" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52285,7 +52282,7 @@
         <v>420</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I17" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52325,7 +52322,7 @@
         <v>429</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I18" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52365,7 +52362,7 @@
         <v>438</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I19" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52405,7 +52402,7 @@
         <v>447</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I20" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52445,7 +52442,7 @@
         <v>458</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I21" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52485,7 +52482,7 @@
         <v>543</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I22" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52525,7 +52522,7 @@
         <v>552</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I23" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52565,7 +52562,7 @@
         <v>561</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I24" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52605,7 +52602,7 @@
         <v>570</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I25" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52645,7 +52642,7 @@
         <v>579</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I26" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52685,7 +52682,7 @@
         <v>467</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I27" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52725,7 +52722,7 @@
         <v>476</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I28" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52765,7 +52762,7 @@
         <v>485</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I29" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52805,7 +52802,7 @@
         <v>494</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I30" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52845,7 +52842,7 @@
         <v>503</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I31" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52885,7 +52882,7 @@
         <v>516</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I32" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52925,7 +52922,7 @@
         <v>525</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I33" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -52965,7 +52962,7 @@
         <v>534</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I34" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53005,7 +53002,7 @@
         <v>590</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I35" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53045,7 +53042,7 @@
         <v>604</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I36" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53085,7 +53082,7 @@
         <v>614</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I37" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53125,7 +53122,7 @@
         <v>623</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I38" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53165,7 +53162,7 @@
         <v>632</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I39" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53205,7 +53202,7 @@
         <v>643</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I40" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53245,7 +53242,7 @@
         <v>657</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I41" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53285,7 +53282,7 @@
         <v>666</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I42" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53325,7 +53322,7 @@
         <v>675</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I43" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53365,7 +53362,7 @@
         <v>686</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I44" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53405,7 +53402,7 @@
         <v>695</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I45" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53445,7 +53442,7 @@
         <v>704</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I46" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53485,7 +53482,7 @@
         <v>713</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I47" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53525,7 +53522,7 @@
         <v>723</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I48" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53565,7 +53562,7 @@
         <v>734</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I49" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53605,7 +53602,7 @@
         <v>744</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I50" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53645,7 +53642,7 @@
         <v>753</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I51" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53685,7 +53682,7 @@
         <v>762</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I52" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53725,7 +53722,7 @@
         <v>773</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I53" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53765,7 +53762,7 @@
         <v>785</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I54" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53805,7 +53802,7 @@
         <v>794</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I55" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53845,7 +53842,7 @@
         <v>807</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I56" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53885,7 +53882,7 @@
         <v>816</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I57" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53925,7 +53922,7 @@
         <v>827</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I58" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -53965,7 +53962,7 @@
         <v>841</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I59" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54005,7 +54002,7 @@
         <v>850</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I60" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54045,7 +54042,7 @@
         <v>861</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I61" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54085,7 +54082,7 @@
         <v>870</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I62" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54125,7 +54122,7 @@
         <v>879</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I63" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54165,7 +54162,7 @@
         <v>888</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I64" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54205,7 +54202,7 @@
         <v>897</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I65" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54245,7 +54242,7 @@
         <v>906</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I66" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54285,7 +54282,7 @@
         <v>915</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I67" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54325,7 +54322,7 @@
         <v>924</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I68" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54365,7 +54362,7 @@
         <v>933</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I69" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54405,7 +54402,7 @@
         <v>59</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I70" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54445,7 +54442,7 @@
         <v>71</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I71" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54485,7 +54482,7 @@
         <v>80</v>
       </c>
       <c r="F72" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I72" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54525,7 +54522,7 @@
         <v>944</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I73" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54565,7 +54562,7 @@
         <v>953</v>
       </c>
       <c r="F74" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I74" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54605,7 +54602,7 @@
         <v>962</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I75" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54645,7 +54642,7 @@
         <v>971</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I76" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54685,7 +54682,7 @@
         <v>980</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I77" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54725,7 +54722,7 @@
         <v>989</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I78" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54765,7 +54762,7 @@
         <v>998</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I79" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54805,7 +54802,7 @@
         <v>1007</v>
       </c>
       <c r="F80" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I80" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54845,7 +54842,7 @@
         <v>1018</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I81" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54885,7 +54882,7 @@
         <v>1028</v>
       </c>
       <c r="F82" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I82" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54925,7 +54922,7 @@
         <v>1037</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I83" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -54965,7 +54962,7 @@
         <v>1049</v>
       </c>
       <c r="F84" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I84" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55005,7 +55002,7 @@
         <v>1058</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I85" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55045,7 +55042,7 @@
         <v>1067</v>
       </c>
       <c r="F86" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I86" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55085,7 +55082,7 @@
         <v>1076</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I87" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55125,7 +55122,7 @@
         <v>1085</v>
       </c>
       <c r="F88" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I88" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55165,7 +55162,7 @@
         <v>1097</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I89" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55205,7 +55202,7 @@
         <v>1106</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I90" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55245,7 +55242,7 @@
         <v>1115</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I91" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55285,7 +55282,7 @@
         <v>1127</v>
       </c>
       <c r="F92" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I92" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55325,7 +55322,7 @@
         <v>1137</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I93" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55365,7 +55362,7 @@
         <v>1147</v>
       </c>
       <c r="F94" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I94" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55405,7 +55402,7 @@
         <v>1156</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I95" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55445,7 +55442,7 @@
         <v>1166</v>
       </c>
       <c r="F96" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I96" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55485,7 +55482,7 @@
         <v>1176</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I97" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55525,7 +55522,7 @@
         <v>1188</v>
       </c>
       <c r="F98" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I98" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55565,7 +55562,7 @@
         <v>1197</v>
       </c>
       <c r="F99" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I99" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55605,7 +55602,7 @@
         <v>1206</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I100" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55645,7 +55642,7 @@
         <v>1215</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I101" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55685,7 +55682,7 @@
         <v>1224</v>
       </c>
       <c r="F102" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I102" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55725,7 +55722,7 @@
         <v>1233</v>
       </c>
       <c r="F103" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I103" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55765,7 +55762,7 @@
         <v>91</v>
       </c>
       <c r="F104" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I104" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55805,7 +55802,7 @@
         <v>102</v>
       </c>
       <c r="F105" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I105" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55845,7 +55842,7 @@
         <v>113</v>
       </c>
       <c r="F106" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I106" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55885,7 +55882,7 @@
         <v>124</v>
       </c>
       <c r="F107" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I107" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55925,7 +55922,7 @@
         <v>133</v>
       </c>
       <c r="F108" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I108" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -55965,7 +55962,7 @@
         <v>144</v>
       </c>
       <c r="F109" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I109" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56005,7 +56002,7 @@
         <v>155</v>
       </c>
       <c r="F110" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I110" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56045,7 +56042,7 @@
         <v>166</v>
       </c>
       <c r="F111" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I111" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56085,7 +56082,7 @@
         <v>175</v>
       </c>
       <c r="F112" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I112" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56125,7 +56122,7 @@
         <v>184</v>
       </c>
       <c r="F113" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I113" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56165,7 +56162,7 @@
         <v>193</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I114" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56205,7 +56202,7 @@
         <v>204</v>
       </c>
       <c r="F115" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I115" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56245,7 +56242,7 @@
         <v>215</v>
       </c>
       <c r="F116" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I116" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56285,7 +56282,7 @@
         <v>228</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I117" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56325,7 +56322,7 @@
         <v>239</v>
       </c>
       <c r="F118" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I118" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56365,7 +56362,7 @@
         <v>248</v>
       </c>
       <c r="F119" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I119" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56405,7 +56402,7 @@
         <v>259</v>
       </c>
       <c r="F120" s="7" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="I120" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"WH_V1")</f>
@@ -56478,10 +56475,10 @@
     <row r="2" ht="26.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="8"/>
       <c r="B2" s="10" t="s">
+        <v>1723</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>1724</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>1725</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>654</v>
@@ -56493,7 +56490,7 @@
         <v>838</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -56519,22 +56516,22 @@
     <row r="3" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
       <c r="B3" s="14" t="s">
+        <v>1726</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>1727</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>1728</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
+        <v>1728</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>1728</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>1729</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>1729</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>1729</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>1730</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
@@ -56560,10 +56557,10 @@
     <row r="4" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
       <c r="B4" s="14" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1731</v>
+        <v>1730</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -56593,13 +56590,13 @@
     <row r="5" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="B5" s="14" t="s">
+        <v>1731</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>1732</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="15" t="s">
         <v>1733</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>1734</v>
       </c>
       <c r="E5" s="15">
         <v>120000</v>
@@ -56634,19 +56631,19 @@
     <row r="6" ht="138" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="14" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="C6" s="14" t="s">
+        <v>1734</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>1735</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="15" t="s">
         <v>1736</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="F6" s="15" t="s">
         <v>1737</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>1738</v>
       </c>
       <c r="G6" s="17">
         <v>65000</v>
@@ -56675,16 +56672,16 @@
     <row r="7" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="14" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="C7" s="14" t="s">
+        <v>1738</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>1739</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E7" s="15" t="s">
         <v>1740</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>1741</v>
       </c>
       <c r="F7" s="15">
         <v>4</v>
@@ -56716,10 +56713,10 @@
     <row r="8" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="14" t="s">
-        <v>1732</v>
+        <v>1731</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1742</v>
+        <v>1741</v>
       </c>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
@@ -56749,10 +56746,10 @@
     <row r="9" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
       <c r="B9" s="14" t="s">
+        <v>1742</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>1743</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>1744</v>
       </c>
       <c r="D9" s="15">
         <v>4500</v>
@@ -56788,19 +56785,19 @@
     <row r="10" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="14" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>1744</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>1745</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>1746</v>
-      </c>
       <c r="E10" s="15" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>1746</v>
+        <v>1745</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
@@ -56827,7 +56824,7 @@
     <row r="11" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="14" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
@@ -56858,19 +56855,19 @@
     <row r="12" ht="87.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
       <c r="B12" s="14" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="C12" s="14" t="s">
+        <v>1746</v>
+      </c>
+      <c r="D12" s="15" t="s">
         <v>1747</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>1748</v>
       </c>
       <c r="E12" s="19">
         <v>0.625</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>1749</v>
+        <v>1748</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -56897,10 +56894,10 @@
     <row r="13" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="B13" s="14" t="s">
-        <v>1743</v>
+        <v>1742</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>1750</v>
+        <v>1749</v>
       </c>
       <c r="D13" s="20">
         <v>0.9</v>
@@ -56936,19 +56933,19 @@
     <row r="14" ht="75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="14" t="s">
+        <v>1750</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>1751</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="15" t="s">
         <v>1752</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="E14" s="15" t="s">
         <v>1753</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="F14" s="18" t="s">
         <v>1754</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>1755</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -56975,19 +56972,19 @@
     <row r="15" ht="262.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="14" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C15" s="14" t="s">
+        <v>1755</v>
+      </c>
+      <c r="D15" s="15" t="s">
         <v>1756</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="E15" s="15" t="s">
         <v>1757</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="F15" s="15" t="s">
         <v>1758</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>1759</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -57014,22 +57011,22 @@
     <row r="16" ht="88.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="14" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C16" s="14" t="s">
+        <v>1759</v>
+      </c>
+      <c r="D16" s="15" t="s">
         <v>1760</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="E16" s="15" t="s">
         <v>1761</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="F16" s="18" t="s">
         <v>1762</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="G16" s="8" t="s">
         <v>1763</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>1764</v>
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -57055,22 +57052,22 @@
     <row r="17" ht="112.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="14" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C17" s="14" t="s">
+        <v>1764</v>
+      </c>
+      <c r="D17" s="15" t="s">
         <v>1765</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="E17" s="15" t="s">
         <v>1766</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="F17" s="15" t="s">
         <v>1767</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="G17" s="8" t="s">
         <v>1768</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>1769</v>
       </c>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -57096,19 +57093,19 @@
     <row r="18" ht="112.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="14" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C18" s="14" t="s">
+        <v>1769</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>1770</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="E18" s="15" t="s">
         <v>1771</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="F18" s="15" t="s">
         <v>1772</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>1773</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -57135,17 +57132,17 @@
     <row r="19" ht="100.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="14" t="s">
-        <v>1751</v>
+        <v>1750</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>1773</v>
+      </c>
+      <c r="D19" s="15" t="s">
         <v>1774</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>1775</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="15" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
@@ -57172,10 +57169,10 @@
     <row r="20" ht="15" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="14" t="s">
+        <v>1776</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>1777</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>1778</v>
       </c>
       <c r="D20" s="20">
         <v>0.95</v>
@@ -57184,7 +57181,7 @@
         <v>0.93</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
@@ -57211,10 +57208,10 @@
     <row r="21" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="14" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>1780</v>
+        <v>1779</v>
       </c>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
@@ -57244,17 +57241,17 @@
     <row r="22" ht="75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="14" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C22" s="14" t="s">
+        <v>1780</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>1781</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>1782</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="15" t="s">
-        <v>1783</v>
+        <v>1782</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
@@ -57281,19 +57278,19 @@
     <row r="23" ht="125.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="14" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C23" s="14" t="s">
+        <v>1783</v>
+      </c>
+      <c r="D23" s="15" t="s">
         <v>1784</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="E23" s="15" t="s">
         <v>1785</v>
       </c>
-      <c r="E23" s="15" t="s">
-        <v>1786</v>
-      </c>
       <c r="F23" s="15" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
@@ -57320,10 +57317,10 @@
     <row r="24" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="14" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>1787</v>
+        <v>1786</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
@@ -57353,10 +57350,10 @@
     <row r="25" ht="15" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="14" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
@@ -57386,19 +57383,19 @@
     <row r="26" ht="87.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="14" t="s">
+        <v>1788</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>1789</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="D26" s="15" t="s">
         <v>1790</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="E26" s="15" t="s">
         <v>1791</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="F26" s="15" t="s">
         <v>1792</v>
-      </c>
-      <c r="F26" s="15" t="s">
-        <v>1793</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
@@ -57425,19 +57422,19 @@
     <row r="27" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C27" s="14" t="s">
+        <v>1793</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>1794</v>
       </c>
-      <c r="D27" s="15" t="s">
-        <v>1795</v>
-      </c>
       <c r="E27" s="15" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
@@ -57464,19 +57461,19 @@
     <row r="28" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C28" s="14" t="s">
+        <v>1795</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>1796</v>
       </c>
-      <c r="D28" s="15" t="s">
-        <v>1797</v>
-      </c>
       <c r="E28" s="15" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>1797</v>
+        <v>1796</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
@@ -57503,10 +57500,10 @@
     <row r="29" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>1798</v>
+        <v>1797</v>
       </c>
       <c r="D29" s="15">
         <v>4</v>
@@ -57542,16 +57539,16 @@
     <row r="30" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>1799</v>
+        <v>1798</v>
       </c>
       <c r="D30" s="18">
         <v>10</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="F30" s="15">
         <v>8</v>
@@ -57581,17 +57578,17 @@
     <row r="31" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31" s="13"/>
       <c r="B31" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="15" t="s">
+        <v>1801</v>
+      </c>
+      <c r="F31" s="15" t="s">
         <v>1802</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>1803</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -57618,19 +57615,19 @@
     <row r="32" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>
       <c r="B32" s="14" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
       <c r="C32" s="14" t="s">
+        <v>1803</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>1804</v>
       </c>
-      <c r="D32" s="15" t="s">
-        <v>1805</v>
-      </c>
       <c r="E32" s="15" t="s">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
@@ -57657,17 +57654,17 @@
     <row r="33" ht="162.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33" s="13"/>
       <c r="B33" s="14" t="s">
+        <v>1805</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>1806</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="D33" s="15" t="s">
         <v>1807</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>1808</v>
       </c>
       <c r="E33" s="16"/>
       <c r="F33" s="15" t="s">
-        <v>1809</v>
+        <v>1808</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
@@ -57694,10 +57691,10 @@
     <row r="34" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34" s="13"/>
       <c r="B34" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>1810</v>
+        <v>1809</v>
       </c>
       <c r="D34" s="16"/>
       <c r="E34" s="16"/>
@@ -57727,19 +57724,19 @@
     <row r="35" ht="237.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35" s="13"/>
       <c r="B35" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C35" s="14" t="s">
+        <v>1810</v>
+      </c>
+      <c r="D35" s="15" t="s">
         <v>1811</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>1812</v>
       </c>
-      <c r="E35" s="15" t="s">
+      <c r="F35" s="15" t="s">
         <v>1813</v>
-      </c>
-      <c r="F35" s="15" t="s">
-        <v>1814</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
@@ -57766,13 +57763,13 @@
     <row r="36" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36" s="13"/>
       <c r="B36" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C36" s="14" t="s">
+        <v>1814</v>
+      </c>
+      <c r="D36" s="15" t="s">
         <v>1815</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>1816</v>
       </c>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
@@ -57801,19 +57798,19 @@
     <row r="37" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37" s="13"/>
       <c r="B37" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C37" s="14" t="s">
+        <v>1816</v>
+      </c>
+      <c r="D37" s="15" t="s">
         <v>1817</v>
       </c>
-      <c r="D37" s="15" t="s">
+      <c r="E37" s="15" t="s">
         <v>1818</v>
       </c>
-      <c r="E37" s="15" t="s">
-        <v>1819</v>
-      </c>
       <c r="F37" s="22" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
@@ -57840,17 +57837,17 @@
     <row r="38" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38" s="13"/>
       <c r="B38" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C38" s="14" t="s">
+        <v>1819</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>1820</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>1821</v>
       </c>
       <c r="E38" s="16"/>
       <c r="F38" s="15" t="s">
-        <v>1822</v>
+        <v>1821</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
@@ -57877,17 +57874,17 @@
     <row r="39" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39" s="13"/>
       <c r="B39" s="14" t="s">
-        <v>1806</v>
+        <v>1805</v>
       </c>
       <c r="C39" s="14" t="s">
+        <v>1822</v>
+      </c>
+      <c r="D39" s="15" t="s">
         <v>1823</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>1824</v>
       </c>
       <c r="E39" s="16"/>
       <c r="F39" s="15" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
@@ -57919,16 +57916,16 @@
         <v>164</v>
       </c>
       <c r="C40" s="14" t="s">
+        <v>1824</v>
+      </c>
+      <c r="D40" s="15" t="s">
         <v>1825</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="E40" s="15" t="s">
         <v>1826</v>
       </c>
-      <c r="E40" s="15" t="s">
+      <c r="F40" s="15" t="s">
         <v>1827</v>
-      </c>
-      <c r="F40" s="15" t="s">
-        <v>1828</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
@@ -57960,7 +57957,7 @@
         <v>164</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>1829</v>
+        <v>1828</v>
       </c>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
@@ -57993,16 +57990,16 @@
         <v>164</v>
       </c>
       <c r="C42" s="14" t="s">
+        <v>1829</v>
+      </c>
+      <c r="D42" s="15" t="s">
         <v>1830</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="E42" s="15" t="s">
         <v>1831</v>
       </c>
-      <c r="E42" s="15" t="s">
+      <c r="F42" s="18" t="s">
         <v>1832</v>
-      </c>
-      <c r="F42" s="18" t="s">
-        <v>1833</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
@@ -58032,7 +58029,7 @@
         <v>164</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>1798</v>
+        <v>1797</v>
       </c>
       <c r="D43" s="15">
         <v>4</v>
@@ -58071,7 +58068,7 @@
         <v>164</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>1834</v>
+        <v>1833</v>
       </c>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>
@@ -58104,7 +58101,7 @@
         <v>164</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>1835</v>
+        <v>1834</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16"/>
@@ -58137,7 +58134,7 @@
         <v>164</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>1836</v>
+        <v>1835</v>
       </c>
       <c r="D46" s="16"/>
       <c r="E46" s="16"/>
@@ -58170,16 +58167,16 @@
         <v>164</v>
       </c>
       <c r="C47" s="14" t="s">
+        <v>1836</v>
+      </c>
+      <c r="D47" s="15" t="s">
         <v>1837</v>
       </c>
-      <c r="D47" s="15" t="s">
+      <c r="E47" s="15" t="s">
         <v>1838</v>
       </c>
-      <c r="E47" s="15" t="s">
-        <v>1839</v>
-      </c>
       <c r="F47" s="15" t="s">
-        <v>1839</v>
+        <v>1838</v>
       </c>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
@@ -58206,19 +58203,19 @@
     <row r="48" ht="150" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A48" s="13"/>
       <c r="B48" s="14" t="s">
+        <v>1839</v>
+      </c>
+      <c r="C48" s="14" t="s">
         <v>1840</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="D48" s="15" t="s">
         <v>1841</v>
       </c>
-      <c r="D48" s="15" t="s">
+      <c r="E48" s="15" t="s">
         <v>1842</v>
       </c>
-      <c r="E48" s="15" t="s">
+      <c r="F48" s="15" t="s">
         <v>1843</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>1844</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
@@ -58245,19 +58242,19 @@
     <row r="49" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A49" s="13"/>
       <c r="B49" s="14" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="C49" s="14" t="s">
+        <v>1844</v>
+      </c>
+      <c r="D49" s="15" t="s">
         <v>1845</v>
       </c>
-      <c r="D49" s="15" t="s">
+      <c r="E49" s="15" t="s">
         <v>1846</v>
       </c>
-      <c r="E49" s="15" t="s">
-        <v>1847</v>
-      </c>
       <c r="F49" s="15" t="s">
-        <v>1847</v>
+        <v>1846</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
@@ -58284,10 +58281,10 @@
     <row r="50" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50" s="13"/>
       <c r="B50" s="14" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>1848</v>
+        <v>1847</v>
       </c>
       <c r="D50" s="16"/>
       <c r="E50" s="16"/>
@@ -58317,10 +58314,10 @@
     <row r="51" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51" s="13"/>
       <c r="B51" s="14" t="s">
-        <v>1840</v>
+        <v>1839</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
       <c r="D51" s="16"/>
       <c r="E51" s="16"/>
@@ -58353,7 +58350,7 @@
         <v>257</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
       <c r="D52" s="16"/>
       <c r="E52" s="16"/>
@@ -58386,10 +58383,10 @@
         <v>257</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
       <c r="E53" s="16"/>
       <c r="F53" s="16"/>
@@ -58421,14 +58418,14 @@
         <v>257</v>
       </c>
       <c r="C54" s="14" t="s">
+        <v>1851</v>
+      </c>
+      <c r="D54" s="15" t="s">
         <v>1852</v>
-      </c>
-      <c r="D54" s="15" t="s">
-        <v>1853</v>
       </c>
       <c r="E54" s="16"/>
       <c r="F54" s="15" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
@@ -58458,7 +58455,7 @@
         <v>257</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
       <c r="D55" s="16"/>
       <c r="E55" s="16"/>
@@ -58488,13 +58485,13 @@
     <row r="56" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A56" s="13"/>
       <c r="B56" s="14" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C56" s="14" t="s">
+        <v>1755</v>
+      </c>
+      <c r="D56" s="15" t="s">
         <v>1856</v>
-      </c>
-      <c r="C56" s="14" t="s">
-        <v>1756</v>
-      </c>
-      <c r="D56" s="15" t="s">
-        <v>1857</v>
       </c>
       <c r="E56" s="16"/>
       <c r="F56" s="16"/>
@@ -58523,13 +58520,13 @@
     <row r="57" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A57" s="13"/>
       <c r="B57" s="14" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
       <c r="E57" s="16"/>
       <c r="F57" s="16"/>
@@ -58558,16 +58555,16 @@
     <row r="58" ht="187.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A58" s="13"/>
       <c r="B58" s="14" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
       <c r="C58" s="14" t="s">
+        <v>1858</v>
+      </c>
+      <c r="D58" s="15" t="s">
         <v>1859</v>
       </c>
-      <c r="D58" s="15" t="s">
+      <c r="E58" s="15" t="s">
         <v>1860</v>
-      </c>
-      <c r="E58" s="15" t="s">
-        <v>1861</v>
       </c>
       <c r="F58" s="16"/>
       <c r="G58" s="8"/>
@@ -58595,19 +58592,19 @@
     <row r="59" ht="63" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A59" s="13"/>
       <c r="B59" s="14" t="s">
+        <v>1861</v>
+      </c>
+      <c r="C59" s="14" t="s">
         <v>1862</v>
       </c>
-      <c r="C59" s="14" t="s">
+      <c r="D59" s="15" t="s">
         <v>1863</v>
       </c>
-      <c r="D59" s="15" t="s">
+      <c r="E59" s="15" t="s">
         <v>1864</v>
       </c>
-      <c r="E59" s="15" t="s">
+      <c r="F59" s="15" t="s">
         <v>1865</v>
-      </c>
-      <c r="F59" s="15" t="s">
-        <v>1866</v>
       </c>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
@@ -58634,19 +58631,19 @@
     <row r="60" ht="112.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A60" s="13"/>
       <c r="B60" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C60" s="14" t="s">
+        <v>1866</v>
+      </c>
+      <c r="D60" s="15" t="s">
         <v>1867</v>
       </c>
-      <c r="D60" s="15" t="s">
+      <c r="E60" s="15" t="s">
         <v>1868</v>
       </c>
-      <c r="E60" s="15" t="s">
+      <c r="F60" s="15" t="s">
         <v>1869</v>
-      </c>
-      <c r="F60" s="15" t="s">
-        <v>1870</v>
       </c>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
@@ -58673,13 +58670,13 @@
     <row r="61" ht="100.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A61" s="13"/>
       <c r="B61" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C61" s="14" t="s">
+        <v>1870</v>
+      </c>
+      <c r="D61" s="15" t="s">
         <v>1871</v>
-      </c>
-      <c r="D61" s="15" t="s">
-        <v>1872</v>
       </c>
       <c r="E61" s="16"/>
       <c r="F61" s="16"/>
@@ -58708,19 +58705,19 @@
     <row r="62" ht="87.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A62" s="13"/>
       <c r="B62" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>1823</v>
+        <v>1822</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>1873</v>
+        <v>1872</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
@@ -58747,17 +58744,17 @@
     <row r="63" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A63" s="13"/>
       <c r="B63" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>1874</v>
+        <v>1873</v>
       </c>
       <c r="D63" s="16"/>
       <c r="E63" s="15" t="s">
-        <v>1875</v>
+        <v>1874</v>
       </c>
       <c r="F63" s="15" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="G63" s="8"/>
       <c r="H63" s="8"/>
@@ -58784,10 +58781,10 @@
     <row r="64" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A64" s="13"/>
       <c r="B64" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>1876</v>
+        <v>1875</v>
       </c>
       <c r="D64" s="16"/>
       <c r="E64" s="16"/>
@@ -58817,13 +58814,13 @@
     <row r="65" ht="87.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A65" s="13"/>
       <c r="B65" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C65" s="14" t="s">
+        <v>1876</v>
+      </c>
+      <c r="D65" s="15" t="s">
         <v>1877</v>
-      </c>
-      <c r="D65" s="15" t="s">
-        <v>1878</v>
       </c>
       <c r="E65" s="16"/>
       <c r="F65" s="16"/>
@@ -58852,17 +58849,17 @@
     <row r="66" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A66" s="13"/>
       <c r="B66" s="14" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="C66" s="14" t="s">
+        <v>1878</v>
+      </c>
+      <c r="D66" s="15" t="s">
         <v>1879</v>
-      </c>
-      <c r="D66" s="15" t="s">
-        <v>1880</v>
       </c>
       <c r="E66" s="16"/>
       <c r="F66" s="15" t="s">
-        <v>1881</v>
+        <v>1880</v>
       </c>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
@@ -58889,10 +58886,10 @@
     <row r="67" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A67" s="13"/>
       <c r="B67" s="14" t="s">
+        <v>1881</v>
+      </c>
+      <c r="C67" s="14" t="s">
         <v>1882</v>
-      </c>
-      <c r="C67" s="14" t="s">
-        <v>1883</v>
       </c>
       <c r="D67" s="19">
         <v>0.16666666666787933</v>
@@ -58926,10 +58923,10 @@
     <row r="68" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A68" s="13"/>
       <c r="B68" s="16" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
       <c r="C68" s="16" t="s">
-        <v>1884</v>
+        <v>1883</v>
       </c>
       <c r="D68" s="20">
         <v>0.95</v>
@@ -58963,10 +58960,10 @@
     <row r="69" ht="50.25" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A69" s="13"/>
       <c r="B69" s="16" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
       <c r="C69" s="16" t="s">
-        <v>1885</v>
+        <v>1884</v>
       </c>
       <c r="D69" s="20">
         <v>0.02</v>
@@ -58998,13 +58995,13 @@
     <row r="70" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A70" s="13"/>
       <c r="B70" s="16" t="s">
-        <v>1882</v>
+        <v>1881</v>
       </c>
       <c r="C70" s="16" t="s">
+        <v>1885</v>
+      </c>
+      <c r="D70" s="15" t="s">
         <v>1886</v>
-      </c>
-      <c r="D70" s="15" t="s">
-        <v>1887</v>
       </c>
       <c r="E70" s="16"/>
       <c r="F70" s="16"/>
@@ -59033,7 +59030,7 @@
     <row r="71" ht="15" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
       <c r="B71" s="16" t="s">
-        <v>1888</v>
+        <v>1887</v>
       </c>
       <c r="C71" s="16"/>
       <c r="D71" s="16"/>
@@ -59064,7 +59061,7 @@
     <row r="72" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A72" s="13"/>
       <c r="B72" s="16" t="s">
-        <v>1889</v>
+        <v>1888</v>
       </c>
       <c r="C72" s="16"/>
       <c r="D72" s="16"/>
@@ -59097,7 +59094,7 @@
     <row r="73" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A73" s="13"/>
       <c r="B73" s="16" t="s">
-        <v>1890</v>
+        <v>1889</v>
       </c>
       <c r="C73" s="16"/>
       <c r="D73" s="16"/>
@@ -59130,7 +59127,7 @@
     <row r="74" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A74" s="13"/>
       <c r="B74" s="16" t="s">
-        <v>1891</v>
+        <v>1890</v>
       </c>
       <c r="C74" s="16"/>
       <c r="D74" s="16"/>
@@ -59161,7 +59158,7 @@
     <row r="75" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A75" s="13"/>
       <c r="B75" s="16" t="s">
-        <v>1892</v>
+        <v>1891</v>
       </c>
       <c r="C75" s="16"/>
       <c r="D75" s="16"/>
@@ -59192,7 +59189,7 @@
     <row r="76" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A76" s="13"/>
       <c r="B76" s="16" t="s">
-        <v>1893</v>
+        <v>1892</v>
       </c>
       <c r="C76" s="16"/>
       <c r="D76" s="16"/>
@@ -59223,7 +59220,7 @@
     <row r="77" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A77" s="13"/>
       <c r="B77" s="16" t="s">
-        <v>1894</v>
+        <v>1893</v>
       </c>
       <c r="C77" s="16"/>
       <c r="D77" s="16"/>
@@ -59254,7 +59251,7 @@
     <row r="78" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A78" s="13"/>
       <c r="B78" s="16" t="s">
-        <v>1895</v>
+        <v>1894</v>
       </c>
       <c r="C78" s="16"/>
       <c r="D78" s="16"/>
@@ -59285,7 +59282,7 @@
     <row r="79" ht="15" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
       <c r="B79" s="16" t="s">
-        <v>1896</v>
+        <v>1895</v>
       </c>
       <c r="C79" s="16"/>
       <c r="D79" s="16"/>
@@ -59316,7 +59313,7 @@
     <row r="80" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A80" s="13"/>
       <c r="B80" s="16" t="s">
-        <v>1897</v>
+        <v>1896</v>
       </c>
       <c r="C80" s="16"/>
       <c r="D80" s="16"/>
@@ -59347,7 +59344,7 @@
     <row r="81" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A81" s="13"/>
       <c r="B81" s="16" t="s">
-        <v>1898</v>
+        <v>1897</v>
       </c>
       <c r="C81" s="16"/>
       <c r="D81" s="16"/>
@@ -59378,7 +59375,7 @@
     <row r="82" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A82" s="13"/>
       <c r="B82" s="16" t="s">
-        <v>1899</v>
+        <v>1898</v>
       </c>
       <c r="C82" s="16"/>
       <c r="D82" s="16"/>
@@ -59409,7 +59406,7 @@
     <row r="83" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A83" s="13"/>
       <c r="B83" s="16" t="s">
-        <v>1900</v>
+        <v>1899</v>
       </c>
       <c r="C83" s="16"/>
       <c r="D83" s="16"/>
@@ -59440,7 +59437,7 @@
     <row r="84" ht="37.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A84" s="13"/>
       <c r="B84" s="16" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="C84" s="16"/>
       <c r="D84" s="16"/>
@@ -59471,7 +59468,7 @@
     <row r="85" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A85" s="13"/>
       <c r="B85" s="16" t="s">
-        <v>1901</v>
+        <v>1900</v>
       </c>
       <c r="C85" s="16"/>
       <c r="D85" s="16"/>
@@ -59502,7 +59499,7 @@
     <row r="86" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A86" s="13"/>
       <c r="B86" s="16" t="s">
-        <v>1902</v>
+        <v>1901</v>
       </c>
       <c r="C86" s="16"/>
       <c r="D86" s="16"/>
@@ -59533,7 +59530,7 @@
     <row r="87" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A87" s="13"/>
       <c r="B87" s="16" t="s">
-        <v>1903</v>
+        <v>1902</v>
       </c>
       <c r="C87" s="16"/>
       <c r="D87" s="16"/>
@@ -59564,7 +59561,7 @@
     <row r="88" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A88" s="13"/>
       <c r="B88" s="16" t="s">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="C88" s="16"/>
       <c r="D88" s="16"/>
@@ -59595,7 +59592,7 @@
     <row r="89" ht="25.5" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A89" s="13"/>
       <c r="B89" s="16" t="s">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="C89" s="16"/>
       <c r="D89" s="16"/>
@@ -59887,10 +59884,10 @@
     <row r="99" ht="24.75" customHeight="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A99" s="8"/>
       <c r="B99" s="23" t="s">
+        <v>1905</v>
+      </c>
+      <c r="C99" s="23" t="s">
         <v>1906</v>
-      </c>
-      <c r="C99" s="23" t="s">
-        <v>1907</v>
       </c>
       <c r="D99" s="23"/>
       <c r="E99" s="23"/>

</xml_diff>